<commit_message>
First version of the Java 26 article
</commit_message>
<xml_diff>
--- a/_drafts/jep-overview.xlsx
+++ b/_drafts/jep-overview.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hanno/Code/websites/hanno.codes/_drafts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172BF6F0-7D86-A642-A3C6-B3304148649C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A6B6B7-7EDC-0D46-9734-240FCF239632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21580" xr2:uid="{D428FD44-A7BE-744F-BBBE-F876344939DC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{D428FD44-A7BE-744F-BBBE-F876344939DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="86">
   <si>
     <t>Status</t>
   </si>
@@ -248,9 +248,6 @@
     <t>Removal</t>
   </si>
   <si>
-    <t>Changes since Java 24</t>
-  </si>
-  <si>
     <t>HotSpot / JFR</t>
   </si>
   <si>
@@ -264,6 +261,42 @@
   </si>
   <si>
     <t>New API</t>
+  </si>
+  <si>
+    <t>Prepare to Make Final Mean Final</t>
+  </si>
+  <si>
+    <t>Remove the Applet API</t>
+  </si>
+  <si>
+    <t>Ahead-of-Time Object Caching with Any GC</t>
+  </si>
+  <si>
+    <t>HTTP 3 for the HTTP Client API</t>
+  </si>
+  <si>
+    <t>G1 GC Improve Throughput by Reducing Synchronization</t>
+  </si>
+  <si>
+    <t>Sixth Preview</t>
+  </si>
+  <si>
+    <t>Lazy Constants</t>
+  </si>
+  <si>
+    <t>Eleventh Incubator</t>
+  </si>
+  <si>
+    <t>Changes since previous Java version</t>
+  </si>
+  <si>
+    <t>Client Libs</t>
+  </si>
+  <si>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>Warnings</t>
   </si>
 </sst>
 </file>
@@ -650,21 +683,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3052CF8C-A168-7D4A-AD88-5F8C700EAEB4}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
     <col min="2" max="2" width="4.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40.5" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
@@ -682,7 +715,7 @@
         <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>51</v>
@@ -738,7 +771,7 @@
         <v>46</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H43" si="0">"### JEP "&amp;B3&amp;": "&amp;C3&amp;IF(D3&lt;&gt;""," ("&amp;D3&amp;")","")</f>
+        <f t="shared" ref="H3:H53" si="0">"### JEP "&amp;B3&amp;": "&amp;C3&amp;IF(D3&lt;&gt;""," ("&amp;D3&amp;")","")</f>
         <v>### JEP 450: Compact Object Headers (Experimental)</v>
       </c>
     </row>
@@ -1083,7 +1116,7 @@
         <v>21</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>45</v>
@@ -1294,7 +1327,7 @@
         <v>### JEP 501: Deprecate the 32-bit x86 Port for Removal</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1321,7 +1354,7 @@
         <v>### JEP 470: PEM Encodings of Cryptographic Objects (Preview)</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>25</v>
       </c>
@@ -1338,7 +1371,7 @@
         <v>38</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>46</v>
@@ -1348,7 +1381,7 @@
         <v>### JEP 502: Stable Values (Preview)</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>25</v>
       </c>
@@ -1372,7 +1405,7 @@
         <v>### JEP 503: Remove the 32-bit x86 Port</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>25</v>
       </c>
@@ -1399,7 +1432,7 @@
         <v>### JEP 505: Structured Concurrency (Fifth Preview)</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>25</v>
       </c>
@@ -1423,7 +1456,7 @@
         <v>### JEP 506: Scoped Values</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>25</v>
       </c>
@@ -1450,7 +1483,7 @@
         <v>### JEP 507: Primitive Types in Patterns, instanceof, and switch (Third Preview)</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>25</v>
       </c>
@@ -1467,7 +1500,7 @@
         <v>15</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>44</v>
@@ -1477,7 +1510,7 @@
         <v>### JEP 508: Vector API (Tenth Incubator)</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>25</v>
       </c>
@@ -1491,10 +1524,10 @@
         <v>6</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>46</v>
@@ -1504,7 +1537,7 @@
         <v>### JEP 509: JFR CPU-Time Profiling (Experimental)</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>25</v>
       </c>
@@ -1528,7 +1561,7 @@
         <v>### JEP 510: Key Derivation Function API</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>25</v>
       </c>
@@ -1552,7 +1585,7 @@
         <v>### JEP 511: Module Import Declarations</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>25</v>
       </c>
@@ -1576,7 +1609,7 @@
         <v>### JEP 512: Compact Source Files and Instance Main Methods</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>25</v>
       </c>
@@ -1600,7 +1633,7 @@
         <v>### JEP 513: Flexible Constructor Bodies</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>25</v>
       </c>
@@ -1624,7 +1657,7 @@
         <v>### JEP 514: Ahead-of-Time Command-Line Ergonomics</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>25</v>
       </c>
@@ -1648,7 +1681,7 @@
         <v>### JEP 515: Ahead-of-Time Method Profiling</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>25</v>
       </c>
@@ -1659,10 +1692,10 @@
         <v>66</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>46</v>
@@ -1672,7 +1705,7 @@
         <v>### JEP 518: JFR Cooperative Sampling</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>25</v>
       </c>
@@ -1696,7 +1729,7 @@
         <v>### JEP 519: Compact Object Headers</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>25</v>
       </c>
@@ -1707,10 +1740,10 @@
         <v>67</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>46</v>
@@ -1720,7 +1753,7 @@
         <v>### JEP 520: JFR Method Timing &amp; Tracing</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>25</v>
       </c>
@@ -1737,18 +1770,273 @@
         <v>42</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H43" t="str">
         <f t="shared" si="0"/>
         <v>### JEP 521: Generational Shenandoah</v>
       </c>
     </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>26</v>
+      </c>
+      <c r="B44">
+        <v>500</v>
+      </c>
+      <c r="C44" t="s">
+        <v>74</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H44" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 500: Prepare to Make Final Mean Final</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>26</v>
+      </c>
+      <c r="B45">
+        <v>504</v>
+      </c>
+      <c r="C45" t="s">
+        <v>75</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H45" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 504: Remove the Applet API</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>26</v>
+      </c>
+      <c r="B46">
+        <v>516</v>
+      </c>
+      <c r="C46" t="s">
+        <v>76</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H46" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 516: Ahead-of-Time Object Caching with Any GC</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>26</v>
+      </c>
+      <c r="B47">
+        <v>517</v>
+      </c>
+      <c r="C47" t="s">
+        <v>77</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H47" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 517: HTTP 3 for the HTTP Client API</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>26</v>
+      </c>
+      <c r="B48">
+        <v>522</v>
+      </c>
+      <c r="C48" t="s">
+        <v>78</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H48" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 522: G1 GC Improve Throughput by Reducing Synchronization</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>26</v>
+      </c>
+      <c r="B49">
+        <v>524</v>
+      </c>
+      <c r="C49" t="s">
+        <v>56</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H49" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 524: PEM Encodings of Cryptographic Objects (Second Preview)</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>26</v>
+      </c>
+      <c r="B50">
+        <v>525</v>
+      </c>
+      <c r="C50" t="s">
+        <v>30</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H50" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 525: Structured Concurrency (Sixth Preview)</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>26</v>
+      </c>
+      <c r="B51">
+        <v>526</v>
+      </c>
+      <c r="C51" t="s">
+        <v>80</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H51" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 526: Lazy Constants (Second Preview)</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>26</v>
+      </c>
+      <c r="B52">
+        <v>529</v>
+      </c>
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H52" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 529: Vector API (Eleventh Incubator)</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>26</v>
+      </c>
+      <c r="B53">
+        <v>530</v>
+      </c>
+      <c r="C53" t="s">
+        <v>60</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H53" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 530: Primitive Types in Patterns, instanceof, and switch (Fourth Preview)</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G43" xr:uid="{3052CF8C-A168-7D4A-AD88-5F8C700EAEB4}">
+  <autoFilter ref="A1:G53" xr:uid="{3052CF8C-A168-7D4A-AD88-5F8C700EAEB4}">
     <filterColumn colId="0">
       <filters>
-        <filter val="25"/>
+        <filter val="26"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
1st version of Java 27 article
</commit_message>
<xml_diff>
--- a/_drafts/jep-overview.xlsx
+++ b/_drafts/jep-overview.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hanno/Code/websites/hanno.codes/_drafts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A6B6B7-7EDC-0D46-9734-240FCF239632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33736F07-44D8-7D4F-A632-971275E48040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{D428FD44-A7BE-744F-BBBE-F876344939DC}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="93">
   <si>
     <t>Status</t>
   </si>
@@ -297,6 +297,27 @@
   </si>
   <si>
     <t>Warnings</t>
+  </si>
+  <si>
+    <t>Make G1 the Default Garbage Collector in All Environments</t>
+  </si>
+  <si>
+    <t>Post-Quantum Hybrid Key Exchange for TLS 1.3</t>
+  </si>
+  <si>
+    <t>Seventh Preview</t>
+  </si>
+  <si>
+    <t>Compact Object Headers by Default</t>
+  </si>
+  <si>
+    <t>JFR In-Process Data Redaction</t>
+  </si>
+  <si>
+    <t>Twelfth Incubator</t>
+  </si>
+  <si>
+    <t>New default</t>
   </si>
 </sst>
 </file>
@@ -683,16 +704,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3052CF8C-A168-7D4A-AD88-5F8C700EAEB4}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.5" customWidth="1"/>
-    <col min="4" max="4" width="16.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="21" style="2" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="33.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -771,7 +792,7 @@
         <v>46</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H53" si="0">"### JEP "&amp;B3&amp;": "&amp;C3&amp;IF(D3&lt;&gt;""," ("&amp;D3&amp;")","")</f>
+        <f t="shared" ref="H3:H62" si="0">"### JEP "&amp;B3&amp;": "&amp;C3&amp;IF(D3&lt;&gt;""," ("&amp;D3&amp;")","")</f>
         <v>### JEP 450: Compact Object Headers (Experimental)</v>
       </c>
     </row>
@@ -1777,7 +1798,7 @@
         <v>### JEP 521: Generational Shenandoah</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>26</v>
       </c>
@@ -1801,7 +1822,7 @@
         <v>### JEP 500: Prepare to Make Final Mean Final</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>26</v>
       </c>
@@ -1825,7 +1846,7 @@
         <v>### JEP 504: Remove the Applet API</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>26</v>
       </c>
@@ -1849,7 +1870,7 @@
         <v>### JEP 516: Ahead-of-Time Object Caching with Any GC</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>26</v>
       </c>
@@ -1873,7 +1894,7 @@
         <v>### JEP 517: HTTP 3 for the HTTP Client API</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>26</v>
       </c>
@@ -1897,7 +1918,7 @@
         <v>### JEP 522: G1 GC Improve Throughput by Reducing Synchronization</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>26</v>
       </c>
@@ -1924,7 +1945,7 @@
         <v>### JEP 524: PEM Encodings of Cryptographic Objects (Second Preview)</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>26</v>
       </c>
@@ -1951,7 +1972,7 @@
         <v>### JEP 525: Structured Concurrency (Sixth Preview)</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>26</v>
       </c>
@@ -1978,7 +1999,7 @@
         <v>### JEP 526: Lazy Constants (Second Preview)</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>26</v>
       </c>
@@ -2005,7 +2026,7 @@
         <v>### JEP 529: Vector API (Eleventh Incubator)</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>26</v>
       </c>
@@ -2032,11 +2053,242 @@
         <v>### JEP 530: Primitive Types in Patterns, instanceof, and switch (Fourth Preview)</v>
       </c>
     </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>27</v>
+      </c>
+      <c r="B54">
+        <v>523</v>
+      </c>
+      <c r="C54" t="s">
+        <v>86</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H54" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 523: Make G1 the Default Garbage Collector in All Environments</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>27</v>
+      </c>
+      <c r="B55">
+        <v>527</v>
+      </c>
+      <c r="C55" t="s">
+        <v>87</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H55" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 527: Post-Quantum Hybrid Key Exchange for TLS 1.3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>27</v>
+      </c>
+      <c r="B56">
+        <v>531</v>
+      </c>
+      <c r="C56" t="s">
+        <v>80</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H56" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 531: Lazy Constants (Third Preview)</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>27</v>
+      </c>
+      <c r="B57">
+        <v>532</v>
+      </c>
+      <c r="C57" t="s">
+        <v>60</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H57" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 532: Primitive Types in Patterns, instanceof, and switch (Fifth Preview)</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>27</v>
+      </c>
+      <c r="B58">
+        <v>533</v>
+      </c>
+      <c r="C58" t="s">
+        <v>30</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H58" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 533: Structured Concurrency (Seventh Preview)</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>27</v>
+      </c>
+      <c r="B59">
+        <v>534</v>
+      </c>
+      <c r="C59" t="s">
+        <v>89</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H59" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 534: Compact Object Headers by Default</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>27</v>
+      </c>
+      <c r="B60">
+        <v>536</v>
+      </c>
+      <c r="C60" t="s">
+        <v>90</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H60" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 536: JFR In-Process Data Redaction</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>27</v>
+      </c>
+      <c r="B61">
+        <v>537</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H61" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 537: Vector API (Twelfth Incubator)</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>27</v>
+      </c>
+      <c r="B62">
+        <v>538</v>
+      </c>
+      <c r="C62" t="s">
+        <v>56</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H62" t="str">
+        <f t="shared" si="0"/>
+        <v>### JEP 538: PEM Encodings of Cryptographic Objects (Third Preview)</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G53" xr:uid="{3052CF8C-A168-7D4A-AD88-5F8C700EAEB4}">
+  <autoFilter ref="A1:G62" xr:uid="{3052CF8C-A168-7D4A-AD88-5F8C700EAEB4}">
     <filterColumn colId="0">
       <filters>
-        <filter val="26"/>
+        <filter val="27"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>